<commit_message>
Updated information on the current WP3 model
The data for Annelinn and Aradas has been updated so that the data in mode3 and mode2 is the same as that for Kanaleneiland
</commit_message>
<xml_diff>
--- a/data/s0/Annelinn/archetypes/v2g_behaviour.xlsx
+++ b/data/s0/Annelinn/archetypes/v2g_behaviour.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asier.divasson\Documents\GitHub\CogniCity\data\s0\Annelinn\archetypes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A42678F-E052-41E7-9A34-7625958ED83A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04E0EB0-6135-4AC9-893F-BC13B750A766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plug-in choices" sheetId="3" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="86">
   <si>
     <t xml:space="preserve">Description </t>
   </si>
@@ -185,12 +185,6 @@
     <t>Alternative specific constant for private EV with V2G (EV2G) if the respondent’s current travel mode is public transport.</t>
   </si>
   <si>
-    <t>B_AGE_CSV2G</t>
-  </si>
-  <si>
-    <t>Effect of age (continuous) on choosing carsharing with V2G (CSV2G).</t>
-  </si>
-  <si>
     <t>B_Battery_V2G_allUser</t>
   </si>
   <si>
@@ -251,34 +245,46 @@
     <t>Sensitivity to walking time, applicable to all alternatives and all users.</t>
   </si>
   <si>
-    <t>B_Time_PTBike</t>
-  </si>
-  <si>
-    <t>B_Time_V2G_PTBikeUser</t>
-  </si>
-  <si>
-    <t>B_CAR_OWNERSHIP_V2G</t>
-  </si>
-  <si>
     <t>B_HAVING_KIDS_V2G</t>
   </si>
   <si>
-    <t>B_INCOME_HIGH_V2G</t>
-  </si>
-  <si>
-    <t>Effect of car ownership (owner = 1) on choosing both V2G alternatives (CSV2G and EV2G), relative to non-owners.</t>
-  </si>
-  <si>
     <t>Effect of having children (yes = 1) on choosing both V2G alternatives (CSV2G and EV2G).</t>
   </si>
   <si>
-    <t>Effect of high household income (income &gt; €3000) on choosing both V2G alternatives (CSV2G and EV2G).</t>
-  </si>
-  <si>
-    <t>B_AGE_V2G</t>
-  </si>
-  <si>
-    <t>Effect of age (continuous) on choosing V2G alternatives (CSV2G and EV2G).</t>
+    <t>B_AGE_EV2G</t>
+  </si>
+  <si>
+    <t>Effect of age (continuous) on choosing private EV with V2G (EV2G).</t>
+  </si>
+  <si>
+    <t>B_EV_OWNERSHIP_CSV2G</t>
+  </si>
+  <si>
+    <t>Effect of owning a private EV (EV owner = 1) on choosing carsharing with V2G (CSV2G), relative to non-EV owners.</t>
+  </si>
+  <si>
+    <t>B_EV_OWNERSHIP_EV2G</t>
+  </si>
+  <si>
+    <t>Effect of owning a private EV (EV owner = 1) on choosing private EV with V2G (EV2G), relative to non-EV owners.</t>
+  </si>
+  <si>
+    <t>B_INCOME_LOW_CSV2G</t>
+  </si>
+  <si>
+    <t>Effect of low household income on choosing carsharing with V2G (CSV2G).</t>
+  </si>
+  <si>
+    <t>Sensitivity to minimum guaranteed battery range for V2G alternatives, applicable to all users.</t>
+  </si>
+  <si>
+    <t>B_HAVING_KIDS_CSV2G</t>
+  </si>
+  <si>
+    <t>Effect of having children (yes = 1) on choosing carsharing with V2G (CSV2G).</t>
+  </si>
+  <si>
+    <t>Sensitivity to travel time for V2G alternatives if the current travel mode is public transport or bike.</t>
   </si>
 </sst>
 </file>
@@ -302,18 +308,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -328,10 +328,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -787,10 +788,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.33203125" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.77734375" customWidth="1"/>
     <col min="3" max="3" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
@@ -799,7 +800,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -819,185 +820,191 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>35</v>
       </c>
       <c r="B2" t="s">
         <v>36</v>
       </c>
       <c r="C2">
-        <v>-2.0611999999999999</v>
+        <v>-3.6230000000000002</v>
       </c>
       <c r="D2">
-        <v>0.35249999999999998</v>
+        <v>0.156</v>
       </c>
       <c r="E2">
-        <v>-5.8468999999999998</v>
+        <v>-23.169</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B3" t="s">
         <v>38</v>
       </c>
       <c r="C3">
-        <v>-2.1124000000000001</v>
+        <v>-1.7450000000000001</v>
       </c>
       <c r="D3">
-        <v>0.72160000000000002</v>
+        <v>0.16700000000000001</v>
       </c>
       <c r="E3">
-        <v>-2.9272999999999998</v>
+        <v>-10.458</v>
       </c>
       <c r="F3">
-        <v>3.3999999999999998E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>40</v>
       </c>
       <c r="B4" t="s">
         <v>41</v>
       </c>
       <c r="C4">
-        <v>-2.4081999999999999</v>
+        <v>-1.6619999999999999</v>
       </c>
       <c r="D4">
-        <v>0.21920000000000001</v>
+        <v>0.13500000000000001</v>
       </c>
       <c r="E4">
-        <v>-10.9884</v>
+        <v>-12.32</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B5" t="s">
         <v>43</v>
       </c>
       <c r="C5">
-        <v>-1.8101</v>
+        <v>-1.119</v>
       </c>
       <c r="D5">
-        <v>0.2646</v>
+        <v>0.219</v>
       </c>
       <c r="E5">
-        <v>-6.8414999999999999</v>
+        <v>-5.0999999999999996</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>44</v>
       </c>
       <c r="B6" t="s">
         <v>45</v>
       </c>
       <c r="C6">
-        <v>-1.2776000000000001</v>
+        <v>-2.895</v>
       </c>
       <c r="D6">
-        <v>0.31080000000000002</v>
+        <v>0.16900000000000001</v>
       </c>
       <c r="E6">
-        <v>-4.1101999999999999</v>
+        <v>-17.152999999999999</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B7" t="s">
         <v>47</v>
       </c>
       <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="F7" t="s">
-        <v>39</v>
+        <v>-0.57399999999999995</v>
+      </c>
+      <c r="D7">
+        <v>0.18099999999999999</v>
+      </c>
+      <c r="E7">
+        <v>-3.1680000000000001</v>
+      </c>
+      <c r="F7">
+        <v>2E-3</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>48</v>
       </c>
       <c r="B8" t="s">
         <v>49</v>
       </c>
       <c r="C8">
-        <v>-0.84699999999999998</v>
+        <v>-0.53900000000000003</v>
       </c>
       <c r="D8">
-        <v>0.2135</v>
+        <v>0.14599999999999999</v>
       </c>
       <c r="E8">
-        <v>-3.9674999999999998</v>
+        <v>-3.6869999999999998</v>
       </c>
       <c r="F8">
-        <v>1E-4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>50</v>
       </c>
       <c r="B9" t="s">
         <v>51</v>
       </c>
       <c r="C9">
-        <v>-0.64500000000000002</v>
+        <v>-0.60499999999999998</v>
       </c>
       <c r="D9">
-        <v>0.26140000000000002</v>
+        <v>0.224</v>
       </c>
       <c r="E9">
-        <v>-2.4678</v>
+        <v>-2.6970000000000001</v>
       </c>
       <c r="F9">
-        <v>1.3599999999999999E-2</v>
+        <v>7.0000000000000001E-3</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="D10">
+        <v>2E-3</v>
+      </c>
+      <c r="E10">
+        <v>2.5750000000000002</v>
+      </c>
+      <c r="F10">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>53</v>
-      </c>
-      <c r="C10">
-        <v>-1.44E-2</v>
-      </c>
-      <c r="D10">
-        <v>3.3999999999999998E-3</v>
-      </c>
-      <c r="E10">
-        <v>-4.2594000000000003</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B11" t="s">
-        <v>55</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1007,250 +1014,258 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12">
+        <v>-5.1999999999999998E-2</v>
+      </c>
+      <c r="D12">
+        <v>0.01</v>
+      </c>
+      <c r="E12">
+        <v>-5.0030000000000001</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13">
+        <v>0.48099999999999998</v>
+      </c>
+      <c r="D13">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="E13">
+        <v>5.1559999999999997</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" t="s">
         <v>79</v>
       </c>
-      <c r="C12">
-        <v>0.40189999999999998</v>
-      </c>
-      <c r="D12">
-        <v>0.12379999999999999</v>
-      </c>
-      <c r="E12">
-        <v>3.2452999999999999</v>
-      </c>
-      <c r="F12">
-        <v>1.1999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="C14">
+        <v>0.93899999999999995</v>
+      </c>
+      <c r="D14">
+        <v>9.8000000000000004E-2</v>
+      </c>
+      <c r="E14">
+        <v>9.6310000000000002</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15">
+        <v>-0.27700000000000002</v>
+      </c>
+      <c r="D15">
+        <v>7.6999999999999999E-2</v>
+      </c>
+      <c r="E15">
+        <v>-3.6059999999999999</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16" t="s">
+        <v>81</v>
+      </c>
+      <c r="C16">
+        <v>0.33700000000000002</v>
+      </c>
+      <c r="D16">
+        <v>6.6000000000000003E-2</v>
+      </c>
+      <c r="E16">
+        <v>5.1180000000000003</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B17" t="s">
         <v>57</v>
       </c>
-      <c r="C13">
-        <v>-2.9100000000000001E-2</v>
-      </c>
-      <c r="D13">
-        <v>1.54E-2</v>
-      </c>
-      <c r="E13">
-        <v>-1.8885000000000001</v>
-      </c>
-      <c r="F13">
-        <v>5.8999999999999997E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B14" t="s">
-        <v>80</v>
-      </c>
-      <c r="C14">
-        <v>0.28100000000000003</v>
-      </c>
-      <c r="D14">
-        <v>8.8400000000000006E-2</v>
-      </c>
-      <c r="E14">
-        <v>3.1785999999999999</v>
-      </c>
-      <c r="F14">
-        <v>1.5E-3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B15" t="s">
-        <v>81</v>
-      </c>
-      <c r="C15">
-        <v>0.35299999999999998</v>
-      </c>
-      <c r="D15">
-        <v>9.8799999999999999E-2</v>
-      </c>
-      <c r="E15">
-        <v>3.5737000000000001</v>
-      </c>
-      <c r="F15">
-        <v>4.0000000000000002E-4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+      <c r="C17">
+        <v>-1.4999999999999999E-2</v>
+      </c>
+      <c r="D17">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="E17">
+        <v>-2.2919999999999998</v>
+      </c>
+      <c r="F17">
+        <v>2.1999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B18" t="s">
         <v>59</v>
       </c>
-      <c r="C16">
-        <v>-3.6900000000000002E-2</v>
-      </c>
-      <c r="D16">
-        <v>8.8999999999999999E-3</v>
-      </c>
-      <c r="E16">
-        <v>-4.1360000000000001</v>
-      </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="F18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B19" t="s">
         <v>61</v>
       </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="F17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+      <c r="C19">
+        <v>-2.8000000000000001E-2</v>
+      </c>
+      <c r="D19">
+        <v>1.4E-2</v>
+      </c>
+      <c r="E19">
+        <v>-2.0619999999999998</v>
+      </c>
+      <c r="F19">
+        <v>3.9E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B20" t="s">
         <v>63</v>
       </c>
-      <c r="C18">
-        <v>0.15490000000000001</v>
-      </c>
-      <c r="D18">
-        <v>8.5599999999999996E-2</v>
-      </c>
-      <c r="E18">
-        <v>1.81</v>
-      </c>
-      <c r="F18">
-        <v>7.0300000000000001E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+      <c r="C20">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="D20">
+        <v>2E-3</v>
+      </c>
+      <c r="E20">
+        <v>3.5489999999999999</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B21" t="s">
         <v>65</v>
       </c>
-      <c r="C19">
-        <v>2.5600000000000001E-2</v>
-      </c>
-      <c r="D19">
-        <v>1.2E-2</v>
-      </c>
-      <c r="E19">
-        <v>2.1282000000000001</v>
-      </c>
-      <c r="F19">
-        <v>3.3300000000000003E-2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+      <c r="C21">
+        <v>-2.4E-2</v>
+      </c>
+      <c r="D21">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="E21">
+        <v>-5.319</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B22" t="s">
         <v>67</v>
       </c>
-      <c r="C20">
-        <v>3.5200000000000002E-2</v>
-      </c>
-      <c r="D20">
-        <v>1.1900000000000001E-2</v>
-      </c>
-      <c r="E20">
-        <v>2.9504999999999999</v>
-      </c>
-      <c r="F20">
-        <v>3.2000000000000002E-3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
+      <c r="C22">
+        <v>-5.5E-2</v>
+      </c>
+      <c r="D22">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="E22">
+        <v>-12.738</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B23" t="s">
         <v>69</v>
       </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-      <c r="D21">
-        <v>0.01</v>
-      </c>
-      <c r="E21">
-        <v>1.5</v>
-      </c>
-      <c r="F21" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
+      <c r="C23">
+        <v>-0.151</v>
+      </c>
+      <c r="D23">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="E23">
+        <v>-6.9630000000000001</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B24" t="s">
         <v>71</v>
       </c>
-      <c r="C22">
-        <v>-0.14399999999999999</v>
-      </c>
-      <c r="D22">
-        <v>2.06E-2</v>
-      </c>
-      <c r="E22">
-        <v>-6.9976000000000003</v>
-      </c>
-      <c r="F22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B23" t="s">
-        <v>73</v>
-      </c>
-      <c r="C23">
-        <v>-2.92E-2</v>
-      </c>
-      <c r="D23">
-        <v>4.4000000000000003E-3</v>
-      </c>
-      <c r="E23">
-        <v>-6.6045999999999996</v>
-      </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="2"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="2"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="2"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="2"/>
+      <c r="C24">
+        <v>-3.6999999999999998E-2</v>
+      </c>
+      <c r="D24">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="E24">
+        <v>-10.747999999999999</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1260,7 +1275,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ABED8AC-90DF-4C58-A1F5-329F3BE9A773}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.5546875" bestFit="1" customWidth="1"/>
@@ -1298,13 +1313,13 @@
         <v>36</v>
       </c>
       <c r="C2">
-        <v>-1.7925</v>
+        <v>-3.3290000000000002</v>
       </c>
       <c r="D2">
-        <v>0.40129999999999999</v>
+        <v>0.222</v>
       </c>
       <c r="E2">
-        <v>-4.4664999999999999</v>
+        <v>-15.015000000000001</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1318,16 +1333,16 @@
         <v>38</v>
       </c>
       <c r="C3">
-        <v>-2.1478000000000002</v>
+        <v>-1.871</v>
       </c>
       <c r="D3">
-        <v>0.89990000000000003</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="E3">
-        <v>-2.3868</v>
+        <v>-8.2040000000000006</v>
       </c>
       <c r="F3">
-        <v>1.7000000000000001E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -1338,13 +1353,13 @@
         <v>41</v>
       </c>
       <c r="C4">
-        <v>-2.4283999999999999</v>
+        <v>-1.383</v>
       </c>
       <c r="D4">
-        <v>0.2989</v>
+        <v>0.16400000000000001</v>
       </c>
       <c r="E4">
-        <v>-8.1234999999999999</v>
+        <v>-8.4290000000000003</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -1358,13 +1373,13 @@
         <v>43</v>
       </c>
       <c r="C5">
-        <v>-1.7179</v>
+        <v>-0.97399999999999998</v>
       </c>
       <c r="D5">
-        <v>0.35210000000000002</v>
+        <v>0.26400000000000001</v>
       </c>
       <c r="E5">
-        <v>-4.8784999999999998</v>
+        <v>-3.6869999999999998</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -1372,22 +1387,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" t="s">
         <v>82</v>
       </c>
-      <c r="B6" t="s">
-        <v>83</v>
-      </c>
       <c r="C6">
-        <v>-8.5000000000000006E-3</v>
-      </c>
-      <c r="D6">
-        <v>4.8999999999999998E-3</v>
-      </c>
-      <c r="E6">
-        <v>-1.7238</v>
-      </c>
-      <c r="F6">
-        <v>8.4699999999999998E-2</v>
+        <v>0</v>
+      </c>
+      <c r="F6" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -1398,10 +1407,16 @@
         <v>55</v>
       </c>
       <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="F7" t="s">
-        <v>39</v>
+        <v>-2.5999999999999999E-2</v>
+      </c>
+      <c r="D7">
+        <v>1.2E-2</v>
+      </c>
+      <c r="E7">
+        <v>-2.1240000000000001</v>
+      </c>
+      <c r="F7">
+        <v>3.4000000000000002E-2</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -1409,36 +1424,30 @@
         <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C8">
-        <v>0.55459999999999998</v>
+        <v>0.59399999999999997</v>
       </c>
       <c r="D8">
-        <v>0.17199999999999999</v>
+        <v>0.10299999999999999</v>
       </c>
       <c r="E8">
-        <v>3.2235999999999998</v>
+        <v>5.7869999999999999</v>
       </c>
       <c r="F8">
-        <v>1.2999999999999999E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>83</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>84</v>
       </c>
       <c r="C9">
         <v>0</v>
-      </c>
-      <c r="D9">
-        <v>0.02</v>
-      </c>
-      <c r="E9">
-        <v>-1.05</v>
       </c>
       <c r="F9" t="s">
         <v>39</v>
@@ -1446,42 +1455,42 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C10">
-        <v>0.34910000000000002</v>
+        <v>0.32800000000000001</v>
       </c>
       <c r="D10">
-        <v>0.12670000000000001</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="E10">
-        <v>2.7557</v>
+        <v>3.4129999999999998</v>
       </c>
       <c r="F10">
-        <v>5.8999999999999999E-3</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="B11" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="C11">
-        <v>0.2404</v>
+        <v>-3.1E-2</v>
       </c>
       <c r="D11">
-        <v>0.1381</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="E11">
-        <v>1.7408999999999999</v>
+        <v>-2.0590000000000002</v>
       </c>
       <c r="F11">
-        <v>8.1699999999999995E-2</v>
+        <v>3.9E-2</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1492,10 +1501,16 @@
         <v>63</v>
       </c>
       <c r="C12">
-        <v>0</v>
-      </c>
-      <c r="F12" t="s">
-        <v>39</v>
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="D12">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="E12">
+        <v>2.7440000000000002</v>
+      </c>
+      <c r="F12">
+        <v>6.0000000000000001E-3</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -1506,56 +1521,56 @@
         <v>65</v>
       </c>
       <c r="C13">
-        <v>3.5499999999999997E-2</v>
+        <v>-2.5999999999999999E-2</v>
       </c>
       <c r="D13">
-        <v>1.89E-2</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="E13">
-        <v>1.881</v>
+        <v>-4.6360000000000001</v>
       </c>
       <c r="F13">
-        <v>0.06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="C14">
-        <v>4.0099999999999997E-2</v>
+        <v>-5.1999999999999998E-2</v>
       </c>
       <c r="D14">
-        <v>1.67E-2</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="E14">
-        <v>2.3952</v>
+        <v>-10.468</v>
       </c>
       <c r="F14">
-        <v>1.66E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B15" t="s">
         <v>69</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>-0.13400000000000001</v>
       </c>
       <c r="D15">
-        <v>0.01</v>
+        <v>2.4E-2</v>
       </c>
       <c r="E15">
-        <v>0.41</v>
-      </c>
-      <c r="F15" t="s">
-        <v>39</v>
+        <v>-5.5010000000000003</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -1566,36 +1581,16 @@
         <v>71</v>
       </c>
       <c r="C16">
-        <v>-0.12130000000000001</v>
+        <v>-2.8000000000000001E-2</v>
       </c>
       <c r="D16">
-        <v>2.5999999999999999E-2</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="E16">
-        <v>-4.6745000000000001</v>
+        <v>-5.4980000000000002</v>
       </c>
       <c r="F16">
         <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>72</v>
-      </c>
-      <c r="B17" t="s">
-        <v>73</v>
-      </c>
-      <c r="C17">
-        <v>-2.63E-2</v>
-      </c>
-      <c r="D17">
-        <v>6.7999999999999996E-3</v>
-      </c>
-      <c r="E17">
-        <v>-3.8668</v>
-      </c>
-      <c r="F17">
-        <v>1E-4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>